<commit_message>
Add docs snapshots and update README & index title
Add project UI snapshot images under docs/snapshots and update the Mayzax WBS spreadsheet. Tidy README links and add a reference to the snapshots; also adjust frontend/index.html page title to "Mayzax Recruitment ATS". Files added: multiple PNGs in docs/snapshots. Files modified: README.md, docs/Mayzax_WBS.xlsx, frontend/index.html.
</commit_message>
<xml_diff>
--- a/docs/Mayzax_WBS.xlsx
+++ b/docs/Mayzax_WBS.xlsx
@@ -7,7 +7,7 @@
     <sheet state="visible" name="Auth_Authorization" sheetId="2" r:id="rId6"/>
     <sheet state="visible" name="Recruiter_Management" sheetId="3" r:id="rId7"/>
     <sheet state="visible" name="Client_Management" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Job_Application_Management" sheetId="5" r:id="rId9"/>
+    <sheet state="visible" name="Application_Management" sheetId="5" r:id="rId9"/>
     <sheet state="visible" name="Duplicate_Detection" sheetId="6" r:id="rId10"/>
     <sheet state="visible" name="Analytics_Dashboard" sheetId="7" r:id="rId11"/>
     <sheet state="visible" name="Shift_Logic" sheetId="8" r:id="rId12"/>
@@ -19,9 +19,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="106">
   <si>
-    <t>Module</t>
+    <t>Modules</t>
   </si>
   <si>
     <t>Status</t>
@@ -30,7 +30,7 @@
     <t>Auth_Authorisation</t>
   </si>
   <si>
-    <t>Not Started</t>
+    <t>Done</t>
   </si>
   <si>
     <t>Recruiter_Management</t>
@@ -39,7 +39,7 @@
     <t>Client_Management</t>
   </si>
   <si>
-    <t>Job_Application_Management</t>
+    <t>Application_Management</t>
   </si>
   <si>
     <t>Duplicate_Detection</t>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t>Branding_UI</t>
+  </si>
+  <si>
+    <t>API_Documentation</t>
   </si>
   <si>
     <t>Task</t>
@@ -216,12 +219,6 @@
     <t>UI to paste link and view history</t>
   </si>
   <si>
-    <t>Implement Export Data functionality (Optional)</t>
-  </si>
-  <si>
-    <t>Allow exporting application data to CSV/Excel</t>
-  </si>
-  <si>
     <t>Define Unique Constraints in Database</t>
   </si>
   <si>
@@ -306,12 +303,6 @@
     <t>Ensure dashboard metrics follow shift logic</t>
   </si>
   <si>
-    <t>Write Unit Tests for Shift Logic Service</t>
-  </si>
-  <si>
-    <t>Verify correct date calculation for edge cases</t>
-  </si>
-  <si>
     <t>Verify Shift Logic across all Daily Reports</t>
   </si>
   <si>
@@ -352,7 +343,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd-mm-yyyy"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -375,12 +369,6 @@
       <sz val="13.0"/>
       <color theme="1"/>
       <name val="Roboto"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Montserrat"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -416,7 +404,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -427,19 +415,25 @@
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -504,7 +498,7 @@
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
     </tableStyle>
-    <tableStyle count="3" pivot="0" name="Job_Application_Management-style">
+    <tableStyle count="3" pivot="0" name="Application_Management-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -574,9 +568,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:B9" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:B10" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="2">
-    <tableColumn name="Module" id="1"/>
+    <tableColumn name="Modules" id="1"/>
     <tableColumn name="Status" id="2"/>
   </tableColumns>
   <tableStyleInfo name="Modules-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
@@ -631,7 +625,7 @@
     <tableColumn name="Status" id="4"/>
     <tableColumn name="Completed" id="5"/>
   </tableColumns>
-  <tableStyleInfo name="Job_Application_Management-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Application_Management-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -662,7 +656,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E100" displayName="Table_8" name="Table_8" id="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E99" displayName="Table_8" name="Table_8" id="8">
   <tableColumns count="5">
     <tableColumn name="Task" id="1"/>
     <tableColumn name="Remark" id="2"/>
@@ -889,7 +883,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="34.0"/>
-    <col customWidth="1" min="2" max="2" width="35.13"/>
+    <col customWidth="1" min="2" max="2" width="13.88"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -964,9 +958,17 @@
         <v>3</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B9">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B10">
       <formula1>"Not Started,In Progress,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -974,7 +976,7 @@
     <hyperlink display="Auth_Authorisation" location="Auth_Authorization!A1" ref="A2"/>
     <hyperlink display="Recruiter_Management" location="Recruiter_Management!A1" ref="A3"/>
     <hyperlink display="Client_Management" location="Client_Management!A1" ref="A4"/>
-    <hyperlink display="Job_Application_Management" location="Job_Application_Management!A1" ref="A5"/>
+    <hyperlink display="Application_Management" location="Application_Management!A1" ref="A5"/>
     <hyperlink display="Duplicate_Detection" location="Duplicate_Detection!A1" ref="A6"/>
     <hyperlink display="Analytics_Dashboard" location="Analytics_Dashboard!A1" ref="A7"/>
     <hyperlink display="Shift_Logic" location="Shift_Logic!A1" ref="A8"/>
@@ -994,133 +996,147 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="50.13"/>
-    <col customWidth="1" min="2" max="2" width="37.63"/>
+    <col customWidth="1" min="1" max="1" width="57.13"/>
+    <col customWidth="1" min="2" max="2" width="45.75"/>
     <col customWidth="1" min="3" max="3" width="15.13"/>
     <col customWidth="1" min="4" max="4" width="18.88"/>
-    <col customWidth="1" min="5" max="5" width="12.63"/>
+    <col customWidth="1" min="5" max="5" width="13.5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="s">
+      <c r="E1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="6" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6" t="b">
-        <v>0</v>
+      <c r="E2" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="6" t="s">
+      <c r="B3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="b">
-        <v>0</v>
+      <c r="E3" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="6" t="s">
+      <c r="B4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="b">
-        <v>0</v>
+      <c r="E4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6" t="s">
+      <c r="B5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="7" t="b">
-        <v>0</v>
+      <c r="E5" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6" t="s">
+      <c r="B6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="7" t="b">
-        <v>0</v>
+      <c r="E6" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="6" t="s">
+      <c r="B7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="7" t="b">
-        <v>0</v>
+      <c r="E7" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="6" t="s">
+      <c r="B8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="7" t="b">
-        <v>0</v>
+      <c r="E8" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -8087,133 +8103,147 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="50.13"/>
-    <col customWidth="1" min="2" max="2" width="37.63"/>
+    <col customWidth="1" min="1" max="1" width="50.25"/>
+    <col customWidth="1" min="2" max="2" width="43.13"/>
     <col customWidth="1" min="3" max="3" width="15.13"/>
     <col customWidth="1" min="4" max="4" width="18.88"/>
-    <col customWidth="1" min="5" max="5" width="12.63"/>
+    <col customWidth="1" min="5" max="5" width="13.5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>14</v>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="7" t="b">
-        <v>0</v>
+      <c r="E2" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="6" t="s">
+      <c r="B3" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="b">
-        <v>0</v>
+      <c r="E3" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="6" t="s">
+      <c r="B4" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="b">
-        <v>0</v>
+      <c r="E4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6" t="s">
+      <c r="B5" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="7" t="b">
-        <v>0</v>
+      <c r="E5" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6" t="s">
+      <c r="B6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="7" t="b">
-        <v>0</v>
+      <c r="E6" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="6" t="s">
+      <c r="B7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="7" t="b">
-        <v>0</v>
+      <c r="E7" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="6" t="s">
+      <c r="B8" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="7" t="b">
-        <v>0</v>
+      <c r="E8" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -15180,126 +15210,138 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="50.13"/>
-    <col customWidth="1" min="2" max="2" width="37.63"/>
+    <col customWidth="1" min="1" max="1" width="45.0"/>
+    <col customWidth="1" min="2" max="2" width="54.63"/>
     <col customWidth="1" min="3" max="3" width="15.13"/>
     <col customWidth="1" min="4" max="4" width="18.88"/>
-    <col customWidth="1" min="5" max="5" width="12.63"/>
+    <col customWidth="1" min="5" max="5" width="13.5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>14</v>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="7" t="b">
-        <v>0</v>
+      <c r="E2" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="6" t="s">
+      <c r="B3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="b">
-        <v>0</v>
+      <c r="E3" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="6" t="s">
+      <c r="B4" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="b">
-        <v>0</v>
+      <c r="E4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6" t="s">
+      <c r="B5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="7" t="b">
-        <v>0</v>
+      <c r="E5" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6" t="s">
+      <c r="B6" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="7" t="b">
-        <v>0</v>
+      <c r="E6" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" s="6" t="s">
+      <c r="A7" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="6" t="s">
+      <c r="B7" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="7" t="b">
-        <v>0</v>
+      <c r="E7" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
     </row>
     <row r="9">
       <c r="A9" s="7"/>
@@ -22265,119 +22307,121 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="50.13"/>
-    <col customWidth="1" min="2" max="2" width="37.63"/>
+    <col customWidth="1" min="1" max="1" width="52.63"/>
+    <col customWidth="1" min="2" max="2" width="70.25"/>
     <col customWidth="1" min="3" max="3" width="15.13"/>
     <col customWidth="1" min="4" max="4" width="18.88"/>
-    <col customWidth="1" min="5" max="5" width="12.63"/>
+    <col customWidth="1" min="5" max="5" width="13.5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>14</v>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6" t="s">
+      <c r="B2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="7" t="b">
-        <v>0</v>
+      <c r="E2" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B3" s="6" t="s">
+      <c r="A3" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="6" t="s">
+      <c r="B3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="b">
-        <v>0</v>
+      <c r="E3" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="A4" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="6" t="s">
+      <c r="B4" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="b">
-        <v>0</v>
+      <c r="E4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6" t="s">
+      <c r="B5" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="7" t="b">
-        <v>0</v>
+      <c r="E5" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="A6" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6" t="s">
+      <c r="B6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="7" t="b">
-        <v>0</v>
+      <c r="E6" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" s="7" t="b">
-        <v>0</v>
-      </c>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
     </row>
     <row r="8">
       <c r="A8" s="7"/>
@@ -29332,7 +29376,7 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D7">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D6">
       <formula1>"Not Started,In Progress,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -29350,111 +29394,121 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="50.13"/>
-    <col customWidth="1" min="2" max="2" width="37.63"/>
+    <col customWidth="1" min="1" max="1" width="46.63"/>
+    <col customWidth="1" min="2" max="2" width="52.88"/>
     <col customWidth="1" min="3" max="3" width="15.13"/>
     <col customWidth="1" min="4" max="4" width="18.88"/>
-    <col customWidth="1" min="5" max="5" width="12.63"/>
+    <col customWidth="1" min="5" max="5" width="13.5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>14</v>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6" t="s">
+      <c r="B3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="7" t="b">
-        <v>0</v>
+      <c r="E3" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="B3" s="6" t="s">
+    <row r="4">
+      <c r="A4" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="6" t="s">
+      <c r="B4" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="b">
-        <v>0</v>
+      <c r="E4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" s="6" t="s">
+    <row r="5">
+      <c r="A5" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="6" t="s">
+      <c r="B5" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="b">
-        <v>0</v>
+      <c r="E5" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="6" t="s">
+    <row r="6">
+      <c r="A6" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6" t="s">
+      <c r="B6" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="7" t="b">
-        <v>0</v>
+      <c r="E6" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
     <row r="7">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
     </row>
     <row r="8">
       <c r="A8" s="7"/>
@@ -36427,118 +36481,130 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="50.13"/>
-    <col customWidth="1" min="2" max="2" width="37.63"/>
+    <col customWidth="1" min="1" max="1" width="49.63"/>
+    <col customWidth="1" min="2" max="2" width="44.75"/>
     <col customWidth="1" min="3" max="3" width="15.13"/>
     <col customWidth="1" min="4" max="4" width="18.88"/>
-    <col customWidth="1" min="5" max="5" width="12.63"/>
+    <col customWidth="1" min="5" max="5" width="13.5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>14</v>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6" t="s">
+      <c r="B3" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="7" t="b">
-        <v>0</v>
+      <c r="E3" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B3" s="6" t="s">
+    <row r="4">
+      <c r="A4" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="6" t="s">
+      <c r="B4" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="b">
-        <v>0</v>
+      <c r="E4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B4" s="6" t="s">
+    <row r="5">
+      <c r="A5" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="6" t="s">
+      <c r="B5" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="b">
-        <v>0</v>
+      <c r="E5" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B5" s="6" t="s">
+    <row r="6">
+      <c r="A6" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6" t="s">
+      <c r="B6" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="7" t="b">
-        <v>0</v>
+      <c r="E6" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B6" s="6" t="s">
+    <row r="7">
+      <c r="A7" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6" t="s">
+      <c r="B7" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E7" s="7" t="b">
-        <v>0</v>
+      <c r="E7" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -43512,111 +43578,111 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="50.13"/>
-    <col customWidth="1" min="2" max="2" width="37.63"/>
+    <col customWidth="1" min="1" max="1" width="53.13"/>
+    <col customWidth="1" min="2" max="2" width="47.5"/>
     <col customWidth="1" min="3" max="3" width="15.13"/>
     <col customWidth="1" min="4" max="4" width="18.88"/>
-    <col customWidth="1" min="5" max="5" width="12.63"/>
+    <col customWidth="1" min="5" max="5" width="13.5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>14</v>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6" t="s">
+      <c r="B3" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="7" t="b">
-        <v>0</v>
+      <c r="E3" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="B3" s="6" t="s">
+    <row r="4">
+      <c r="A4" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="6" t="s">
+      <c r="B4" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="6">
+        <v>46206.0</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="b">
-        <v>0</v>
+      <c r="E4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B4" s="6" t="s">
+    <row r="5">
+      <c r="A5" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="6" t="s">
+      <c r="B5" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C5" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="b">
-        <v>0</v>
+      <c r="E5" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="7" t="b">
-        <v>0</v>
-      </c>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
     </row>
     <row r="7">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
     </row>
     <row r="8">
       <c r="A8" s="7"/>
@@ -44263,11 +44329,11 @@
       <c r="E99" s="7"/>
     </row>
     <row r="100">
-      <c r="A100" s="7"/>
-      <c r="B100" s="7"/>
-      <c r="C100" s="7"/>
-      <c r="D100" s="7"/>
-      <c r="E100" s="7"/>
+      <c r="A100" s="8"/>
+      <c r="B100" s="8"/>
+      <c r="C100" s="8"/>
+      <c r="D100" s="8"/>
+      <c r="E100" s="8"/>
     </row>
     <row r="101">
       <c r="A101" s="8"/>
@@ -50562,16 +50628,9 @@
       <c r="D999" s="8"/>
       <c r="E999" s="8"/>
     </row>
-    <row r="1000">
-      <c r="A1000" s="8"/>
-      <c r="B1000" s="8"/>
-      <c r="C1000" s="8"/>
-      <c r="D1000" s="8"/>
-      <c r="E1000" s="8"/>
-    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D6">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D5">
       <formula1>"Not Started,In Progress,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -50589,111 +50648,121 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="50.13"/>
-    <col customWidth="1" min="2" max="2" width="37.63"/>
+    <col customWidth="1" min="1" max="1" width="46.63"/>
+    <col customWidth="1" min="2" max="2" width="52.38"/>
     <col customWidth="1" min="3" max="3" width="15.13"/>
     <col customWidth="1" min="4" max="4" width="18.88"/>
-    <col customWidth="1" min="5" max="5" width="12.63"/>
+    <col customWidth="1" min="5" max="5" width="13.5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>14</v>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C3" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="6" t="s">
+      <c r="B4" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="7" t="b">
-        <v>0</v>
+      <c r="E4" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B3" s="6" t="s">
+    <row r="5">
+      <c r="A5" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="6" t="s">
+      <c r="B5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="b">
-        <v>0</v>
+      <c r="E5" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B4" s="6" t="s">
+    <row r="6">
+      <c r="A6" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="6" t="s">
+      <c r="B6" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="6">
+        <v>46207.0</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="7" t="b">
-        <v>0</v>
+      <c r="E6" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="7" t="b">
-        <v>0</v>
-      </c>
-    </row>
     <row r="7">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
     </row>
     <row r="8">
       <c r="A8" s="7"/>

</xml_diff>